<commit_message>
Rename the brand to theCreative.exchange in funding docs and the model
Company name updated in the survey response, positioning memo, market
sizing, fresh-look memo, docs index and the model's README and Comps
sheets. URLs are unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETG5M27XfcTD2TyhhuebtG
</commit_message>
<xml_diff>
--- a/docs/financial-model-5yr-v2.xlsx
+++ b/docs/financial-model-5yr-v2.xlsx
@@ -546,7 +546,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>creatives.exchange — 5-year model v2: two tracks, every revenue source, three scenarios</t>
+          <t>theCreative.exchange — 5-year model v2: two tracks, every revenue source, three scenarios</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>creatives.exchange (this model)</t>
+          <t>theCreative.exchange (this model)</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Update the model and deck for a 5,000-10,000 member three-year SOM
Raise Base organization seat packs (schools, universities, churches,
organizations) so year-three members land at 5,700, inside the founder's
5,000-10,000 estimate. Add the estimate and an inside/below/above check
to the Market sheet. Base revenue moves to $385k in year three and
$1.47M in year five; peak cash need falls from $339k to $286k.

Regenerate the Sankey from the new year-five flows, fix the revenue
headline (creatives and communities keep 90 percent of what they earn),
and update the market, business and ask slides, the fresh-look memo, the
market-sizing doc and the deck README. Remove the team-slide invitation.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETG5M27XfcTD2TyhhuebtG
</commit_message>
<xml_diff>
--- a/docs/financial-model-5yr-v2.xlsx
+++ b/docs/financial-model-5yr-v2.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -169,6 +169,7 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -622,14 +623,14 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>4. Results (computed 2026-09-30). Conservative = a San Diego house community with a few churches: $17k → $264k platform revenue over five years, never breaks even, founder pay $0/$0/$24k. Base = San Diego plus partner communities nationally through the mapped networks, plus organization seats: $36k / $132k / $361k / $777k / $1.42M, cumulative cash need peaks at $339k in Y4, breakeven in Y5, 4,500 members and 31 communities by Y3. Fundable = the Base with a funded team from day one and three metros by Y4: $80k / $310k / $1.0M / $2.4M / $5.3M, profitable in Y3, peak cash need $314k.</t>
+          <t>4. Results (updated 2026-09-30 after raising Base org seat packs to match the founder's 5,000-10,000 member estimate for schools and organizations). Conservative = a San Diego house community with a few churches: $17k → $264k platform revenue over five years, never breaks even, founder pay $0/$0/$24k. Base = San Diego plus partner communities nationally through the mapped networks, plus seats bought by schools, universities, churches and organizations: $36k / $133k / $385k / $810k / $1.47M, cumulative cash need peaks at $286k in Y4, annual EBITDA turns positive in Y5, 5,700 paying and covered members and 31 communities by Y3. Fundable = the Base with a funded team from day one and three metros by Y4: $80k / $310k / $996k / $2.4M / $5.3M, profitable in Y3, peak cash need $314k.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>4b. The market-sizing research (docs/funding/market-sizing.md) says San Diego alone supports about 1,000 paying INDIVIDUAL members in three years. The Conservative case matches that (1,270 paying and covered members in Y3). Everything above it comes from organization seat packs, partner communities outside San Diego, and paid plans, so the Base and Fundable cases are bets on partners, not on San Diego individuals.</t>
+          <t>4b. The market-sizing research (docs/funding/market-sizing.md) says San Diego alone supports about 1,000 paying INDIVIDUAL members in three years; the Conservative case matches that (1,270 paying and covered members in Y3). The founder estimates 5,000-10,000 members in three years once schools, universities, churches and other organizations buy seats (estimate not yet sourced; see the Market sheet). The Base case sits inside that range (5,700 in Y3), Fundable above it (12,700). Note that members are not revenue: an organization-bought seat earns the platform about $10 a year in fees plus the backings and classes its holder buys, so 1,200 extra Base seats added only about $24k of Y3 revenue. Revenue is driven by backing and class volume, partner plans and sponsorships.</t>
         </is>
       </c>
     </row>
@@ -646,7 +647,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>VALUES: this file was built with openpyxl and its formulas were evaluated with a Python formula engine (pycel; 722 formulas, 0 errors in every scenario) because LibreOffice is not available in the build sandbox. Excel and Google Sheets recalculate every formula on open, so what you see is live.</t>
+          <t>VALUES: this file was built with openpyxl and its formulas were evaluated with a Python formula engine (pycel; 724 formulas, 0 errors in every scenario) because LibreOffice is not available in the build sandbox. Excel and Google Sheets recalculate every formula on open, so what you see is live.</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2541,7 @@
       </c>
       <c r="H84" s="8" t="inlineStr">
         <is>
-          <t>Churches and orgs buying seats inside partner communities; platform keeps 10% of these dues</t>
+          <t>Schools, universities, churches and other organizations buying seats for their people; platform keeps 10% of these dues. Base raised 2026-09-30 (Y3 800 to 2,000) to match the founder estimate of 5,000-10,000 members in three years</t>
         </is>
       </c>
     </row>
@@ -2555,16 +2556,16 @@
         <v>0</v>
       </c>
       <c r="D85" s="18" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="E85" s="18" t="n">
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="F85" s="18" t="n">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="H85" s="7" t="n"/>
     </row>
@@ -2605,19 +2606,19 @@
       </c>
       <c r="D87" s="19">
         <f>CHOOSE(Inputs!$B$23,D84,D85,D86)</f>
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="E87" s="19">
         <f>CHOOSE(Inputs!$B$23,E84,E85,E86)</f>
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="F87" s="19">
         <f>CHOOSE(Inputs!$B$23,F84,F85,F86)</f>
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="G87" s="19">
         <f>CHOOSE(Inputs!$B$23,G84,G85,G86)</f>
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="H87" s="7" t="n"/>
     </row>
@@ -5846,19 +5847,19 @@
       </c>
       <c r="C8" s="24">
         <f>Inputs!$D$87</f>
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D8" s="24">
         <f>Inputs!$E$87</f>
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="E8" s="24">
         <f>Inputs!$F$87</f>
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="F8" s="24">
         <f>Inputs!$G$87</f>
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="G8" s="7" t="n"/>
     </row>
@@ -6156,19 +6157,19 @@
       </c>
       <c r="C20" s="27">
         <f>C8*Inputs!$B$17</f>
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="D20" s="27">
         <f>D8*Inputs!$B$17</f>
-        <v>80000</v>
+        <v>200000</v>
       </c>
       <c r="E20" s="27">
         <f>E8*Inputs!$B$17</f>
-        <v>200000</v>
+        <v>350000</v>
       </c>
       <c r="F20" s="27">
         <f>F8*Inputs!$B$17</f>
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="G20" s="7" t="n"/>
     </row>
@@ -6184,19 +6185,19 @@
       </c>
       <c r="C21" s="27">
         <f>(C16+C8)*C10</f>
-        <v>73600</v>
+        <v>81600</v>
       </c>
       <c r="D21" s="27">
         <f>(D16+D8)*D10</f>
-        <v>320000</v>
+        <v>440000</v>
       </c>
       <c r="E21" s="27">
         <f>(E16+E8)*E10</f>
-        <v>960000</v>
+        <v>1140000</v>
       </c>
       <c r="F21" s="27">
         <f>(F16+F8)*F10</f>
-        <v>2240000</v>
+        <v>2520000</v>
       </c>
       <c r="G21" s="7" t="n"/>
     </row>
@@ -6380,19 +6381,19 @@
       </c>
       <c r="C28" s="28">
         <f>SUM(C19:C27)</f>
-        <v>341718.848</v>
+        <v>359718.848</v>
       </c>
       <c r="D28" s="28">
         <f>SUM(D19:D27)</f>
-        <v>1243776.1600000001</v>
+        <v>1483776.1600000001</v>
       </c>
       <c r="E28" s="28">
         <f>SUM(E19:E27)</f>
-        <v>3312190.4</v>
+        <v>3642190.4</v>
       </c>
       <c r="F28" s="28">
         <f>SUM(F19:F27)</f>
-        <v>6998380.8</v>
+        <v>7478380.8</v>
       </c>
       <c r="G28" s="7" t="n"/>
     </row>
@@ -6430,19 +6431,19 @@
       </c>
       <c r="C31" s="27">
         <f>(C19+C20)*Inputs!$B$10</f>
-        <v>10063.8848</v>
+        <v>11063.8848</v>
       </c>
       <c r="D31" s="27">
         <f>(D19+D20)*Inputs!$B$10</f>
-        <v>34879.616</v>
+        <v>46879.61600000001</v>
       </c>
       <c r="E31" s="27">
         <f>(E19+E20)*Inputs!$B$10</f>
-        <v>87199.04000000001</v>
+        <v>102199.04000000001</v>
       </c>
       <c r="F31" s="27">
         <f>(F19+F20)*Inputs!$B$10</f>
-        <v>174398.08000000002</v>
+        <v>194398.08000000002</v>
       </c>
       <c r="G31" s="7" t="n"/>
     </row>
@@ -6458,19 +6459,19 @@
       </c>
       <c r="C32" s="27">
         <f>C21*Inputs!$B$11</f>
-        <v>7360.0</v>
+        <v>8160.0</v>
       </c>
       <c r="D32" s="27">
         <f>D21*Inputs!$B$11</f>
-        <v>32000.0</v>
+        <v>44000.0</v>
       </c>
       <c r="E32" s="27">
         <f>E21*Inputs!$B$11</f>
-        <v>96000.0</v>
+        <v>114000.0</v>
       </c>
       <c r="F32" s="27">
         <f>F21*Inputs!$B$11</f>
-        <v>224000.0</v>
+        <v>252000.0</v>
       </c>
       <c r="G32" s="7" t="n"/>
     </row>
@@ -6654,19 +6655,19 @@
       </c>
       <c r="C39" s="28">
         <f>SUM(C31:C38)</f>
-        <v>60503.8848</v>
+        <v>62303.8848</v>
       </c>
       <c r="D39" s="28">
         <f>SUM(D31:D38)</f>
-        <v>203859.616</v>
+        <v>227859.616</v>
       </c>
       <c r="E39" s="28">
         <f>SUM(E31:E38)</f>
-        <v>514399.04000000004</v>
+        <v>547399.04</v>
       </c>
       <c r="F39" s="28">
         <f>SUM(F31:F38)</f>
-        <v>1042798.0800000001</v>
+        <v>1090798.08</v>
       </c>
       <c r="G39" s="7" t="n"/>
     </row>
@@ -6704,19 +6705,19 @@
       </c>
       <c r="C42" s="27">
         <f>(C19+C20)*(1-Inputs!$B$10)</f>
-        <v>90574.9632</v>
+        <v>99574.9632</v>
       </c>
       <c r="D42" s="27">
         <f>(D19+D20)*(1-Inputs!$B$10)</f>
-        <v>313916.54400000005</v>
+        <v>421916.54400000005</v>
       </c>
       <c r="E42" s="27">
         <f>(E19+E20)*(1-Inputs!$B$10)</f>
-        <v>784791.36</v>
+        <v>919791.36</v>
       </c>
       <c r="F42" s="27">
         <f>(F19+F20)*(1-Inputs!$B$10)</f>
-        <v>1569582.72</v>
+        <v>1749582.72</v>
       </c>
       <c r="G42" s="7" t="n"/>
     </row>
@@ -6732,19 +6733,19 @@
       </c>
       <c r="C43" s="27">
         <f>C21*(1-Inputs!$B$11)+C22*(1-Inputs!$B$12)</f>
-        <v>152640</v>
+        <v>159840</v>
       </c>
       <c r="D43" s="27">
         <f>D21*(1-Inputs!$B$11)+D22*(1-Inputs!$B$12)</f>
-        <v>612000</v>
+        <v>720000</v>
       </c>
       <c r="E43" s="27">
         <f>E21*(1-Inputs!$B$11)+E22*(1-Inputs!$B$12)</f>
-        <v>1728000</v>
+        <v>1890000</v>
       </c>
       <c r="F43" s="27">
         <f>F21*(1-Inputs!$B$11)+F22*(1-Inputs!$B$12)</f>
-        <v>3816000</v>
+        <v>4068000</v>
       </c>
       <c r="G43" s="7" t="n"/>
     </row>
@@ -6838,19 +6839,19 @@
       </c>
       <c r="C48" s="27">
         <f>(C42+C43)*Inputs!$B$22</f>
-        <v>2432.149632</v>
+        <v>2594.149632</v>
       </c>
       <c r="D48" s="27">
         <f>(D42+D43)*Inputs!$B$22</f>
-        <v>9259.16544</v>
+        <v>11419.16544</v>
       </c>
       <c r="E48" s="27">
         <f>(E42+E43)*Inputs!$B$22</f>
-        <v>25127.9136</v>
+        <v>28097.9136</v>
       </c>
       <c r="F48" s="27">
         <f>(F42+F43)*Inputs!$B$22</f>
-        <v>53855.8272</v>
+        <v>58175.8272</v>
       </c>
       <c r="G48" s="7" t="n"/>
     </row>
@@ -6866,19 +6867,19 @@
       </c>
       <c r="C49" s="28">
         <f>C39-C47-C48</f>
-        <v>54281.709312</v>
+        <v>55919.709312</v>
       </c>
       <c r="D49" s="28">
         <f>D39-D47-D48</f>
-        <v>181967.03104</v>
+        <v>203807.03104</v>
       </c>
       <c r="E49" s="28">
         <f>E39-E47-E48</f>
-        <v>457687.5776000001</v>
+        <v>487717.5776000001</v>
       </c>
       <c r="F49" s="28">
         <f>F39-F47-F48</f>
-        <v>925775.1552000002</v>
+        <v>969455.1552000002</v>
       </c>
       <c r="G49" s="7" t="n"/>
     </row>
@@ -6903,19 +6904,19 @@
       </c>
       <c r="C51" s="30">
         <f>IF((C16+C8)=0,0,C39/(C16+C8))</f>
-        <v>65.76509217391305</v>
+        <v>61.08224</v>
       </c>
       <c r="D51" s="30">
         <f>IF((D16+D8)=0,0,D39/(D16+D8))</f>
-        <v>63.70613</v>
+        <v>51.78627636363637</v>
       </c>
       <c r="E51" s="30">
         <f>IF((E16+E8)=0,0,E39/(E16+E8))</f>
-        <v>64.29988</v>
+        <v>57.62095157894737</v>
       </c>
       <c r="F51" s="30">
         <f>IF((F16+F8)=0,0,F39/(F16+F8))</f>
-        <v>65.17488</v>
+        <v>60.599893333333334</v>
       </c>
       <c r="G51" s="7" t="n"/>
     </row>
@@ -6931,19 +6932,19 @@
       </c>
       <c r="C52" s="27">
         <f>IF(C6=0,0,C39/C6)</f>
-        <v>5041.9904</v>
+        <v>5191.9904</v>
       </c>
       <c r="D52" s="27">
         <f>IF(D6=0,0,D39/D6)</f>
-        <v>6795.3205333333335</v>
+        <v>7595.3205333333335</v>
       </c>
       <c r="E52" s="27">
         <f>IF(E6=0,0,E39/E6)</f>
-        <v>8573.317333333334</v>
+        <v>9123.317333333334</v>
       </c>
       <c r="F52" s="27">
         <f>IF(F6=0,0,F39/F6)</f>
-        <v>10427.980800000001</v>
+        <v>10907.980800000001</v>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
@@ -7066,19 +7067,19 @@
       </c>
       <c r="C6" s="26">
         <f>Garden!C27+Exchange!C31</f>
-        <v>45823.5168</v>
+        <v>46823.5168</v>
       </c>
       <c r="D6" s="26">
         <f>Garden!D27+Exchange!D31</f>
-        <v>114758.832</v>
+        <v>126758.83200000001</v>
       </c>
       <c r="E6" s="26">
         <f>Garden!E27+Exchange!E31</f>
-        <v>219557.79200000002</v>
+        <v>234557.79200000002</v>
       </c>
       <c r="F6" s="26">
         <f>Garden!F27+Exchange!F31</f>
-        <v>360876.416</v>
+        <v>380876.416</v>
       </c>
       <c r="G6" s="7" t="n"/>
     </row>
@@ -7094,19 +7095,19 @@
       </c>
       <c r="C7" s="26">
         <f>Garden!C28+Exchange!C32</f>
-        <v>13360</v>
+        <v>14160</v>
       </c>
       <c r="D7" s="26">
         <f>Garden!D28+Exchange!D32</f>
-        <v>48250</v>
+        <v>60250</v>
       </c>
       <c r="E7" s="26">
         <f>Garden!E28+Exchange!E32</f>
-        <v>127500</v>
+        <v>145500</v>
       </c>
       <c r="F7" s="26">
         <f>Garden!F28+Exchange!F32</f>
-        <v>276500</v>
+        <v>304500</v>
       </c>
       <c r="G7" s="7" t="n"/>
     </row>
@@ -7290,19 +7291,19 @@
       </c>
       <c r="C14" s="28">
         <f>SUM(C6:C13)</f>
-        <v>131563.51679999998</v>
+        <v>133363.51679999998</v>
       </c>
       <c r="D14" s="28">
         <f>SUM(D6:D13)</f>
-        <v>361488.832</v>
+        <v>385488.832</v>
       </c>
       <c r="E14" s="28">
         <f>SUM(E6:E13)</f>
-        <v>777207.792</v>
+        <v>810207.792</v>
       </c>
       <c r="F14" s="28">
         <f>SUM(F6:F13)</f>
-        <v>1423776.416</v>
+        <v>1471776.416</v>
       </c>
       <c r="G14" s="7" t="n"/>
     </row>
@@ -7346,19 +7347,19 @@
       </c>
       <c r="C16" s="26">
         <f>Exchange!C39</f>
-        <v>60503.8848</v>
+        <v>62303.8848</v>
       </c>
       <c r="D16" s="26">
         <f>Exchange!D39</f>
-        <v>203859.616</v>
+        <v>227859.616</v>
       </c>
       <c r="E16" s="26">
         <f>Exchange!E39</f>
-        <v>514399.04000000004</v>
+        <v>547399.04</v>
       </c>
       <c r="F16" s="26">
         <f>Exchange!F39</f>
-        <v>1042798.0800000001</v>
+        <v>1090798.08</v>
       </c>
       <c r="G16" s="7" t="n"/>
     </row>
@@ -7374,19 +7375,19 @@
       </c>
       <c r="C17" s="31">
         <f>IF(C14=0,0,(C10+C12+C13)/C14)</f>
-        <v>0.18226937515248912</v>
+        <v>0.17980929549092398</v>
       </c>
       <c r="D17" s="31">
         <f>IF(D14=0,0,(D10+D12+D13)/D14)</f>
-        <v>0.19497144520359622</v>
+        <v>0.18283279345431205</v>
       </c>
       <c r="E17" s="31">
         <f>IF(E14=0,0,(E10+E12+E13)/E14)</f>
-        <v>0.22059737661508158</v>
+        <v>0.21161238103718458</v>
       </c>
       <c r="F17" s="31">
         <f>IF(F14=0,0,(F10+F12+F13)/F14)</f>
-        <v>0.23486833764213721</v>
+        <v>0.2272084240273626</v>
       </c>
       <c r="G17" s="7" t="n"/>
     </row>
@@ -7424,19 +7425,19 @@
       </c>
       <c r="C20" s="26">
         <f>Garden!C24+Exchange!C28</f>
-        <v>631238.112</v>
+        <v>649238.112</v>
       </c>
       <c r="D20" s="26">
         <f>Garden!D24+Exchange!D28</f>
-        <v>1906034.5920000002</v>
+        <v>2146034.592</v>
       </c>
       <c r="E20" s="26">
         <f>Garden!E24+Exchange!E28</f>
-        <v>4478907.904</v>
+        <v>4808907.904</v>
       </c>
       <c r="F20" s="26">
         <f>Garden!F24+Exchange!F28</f>
-        <v>8796337.472</v>
+        <v>9276337.472</v>
       </c>
       <c r="G20" s="7" t="n"/>
     </row>
@@ -7452,19 +7453,19 @@
       </c>
       <c r="C21" s="24">
         <f>Garden!C6+Garden!C7+Exchange!C16+Exchange!C8</f>
-        <v>1520</v>
+        <v>1620</v>
       </c>
       <c r="D21" s="24">
         <f>Garden!D6+Garden!D7+Exchange!D16+Exchange!D8</f>
-        <v>4500</v>
+        <v>5700</v>
       </c>
       <c r="E21" s="24">
         <f>Garden!E6+Garden!E7+Exchange!E16+Exchange!E8</f>
-        <v>10100</v>
+        <v>11600</v>
       </c>
       <c r="F21" s="24">
         <f>Garden!F6+Garden!F7+Exchange!F16+Exchange!F8</f>
-        <v>19000</v>
+        <v>21000</v>
       </c>
       <c r="G21" s="7" t="n"/>
     </row>
@@ -7508,19 +7509,19 @@
       </c>
       <c r="C23" s="26">
         <f>Garden!C19*(1-Inputs!$B$11)+Garden!C20*(1-Inputs!$B$12)+Garden!C38+Exchange!C43+Exchange!C44</f>
-        <v>357599.632</v>
+        <v>364799.632</v>
       </c>
       <c r="D23" s="26">
         <f>Garden!D19*(1-Inputs!$B$11)+Garden!D20*(1-Inputs!$B$12)+Garden!D38+Exchange!D43+Exchange!D44</f>
-        <v>1117129.216</v>
+        <v>1225129.216</v>
       </c>
       <c r="E23" s="26">
         <f>Garden!E19*(1-Inputs!$B$11)+Garden!E20*(1-Inputs!$B$12)+Garden!E38+Exchange!E43+Exchange!E44</f>
-        <v>2685658.752</v>
+        <v>2847658.752</v>
       </c>
       <c r="F23" s="26">
         <f>Garden!F19*(1-Inputs!$B$11)+Garden!F20*(1-Inputs!$B$12)+Garden!F38+Exchange!F43+Exchange!F44</f>
-        <v>5392978.336</v>
+        <v>5644978.336</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
@@ -7540,19 +7541,19 @@
       </c>
       <c r="C24" s="30">
         <f>IF(C21=0,0,C14/C21)</f>
-        <v>86.55494526315789</v>
+        <v>82.32315851851851</v>
       </c>
       <c r="D24" s="30">
         <f>IF(D21=0,0,D14/D21)</f>
-        <v>80.33085155555555</v>
+        <v>67.6296196491228</v>
       </c>
       <c r="E24" s="30">
         <f>IF(E21=0,0,E14/E21)</f>
-        <v>76.95126653465347</v>
+        <v>69.84549931034483</v>
       </c>
       <c r="F24" s="30">
         <f>IF(F21=0,0,F14/F21)</f>
-        <v>74.93560084210526</v>
+        <v>70.08459123809524</v>
       </c>
       <c r="G24" s="7" t="n"/>
     </row>
@@ -7568,19 +7569,19 @@
       </c>
       <c r="C25" s="31">
         <f>IF(C20=0,0,C14/C20)</f>
-        <v>0.20842137744686745</v>
+        <v>0.2054154159083008</v>
       </c>
       <c r="D25" s="31">
         <f>IF(D20=0,0,D14/D20)</f>
-        <v>0.18965491681905422</v>
+        <v>0.17962843350103835</v>
       </c>
       <c r="E25" s="31">
         <f>IF(E20=0,0,E14/E20)</f>
-        <v>0.1735261828683495</v>
+        <v>0.16848062141636722</v>
       </c>
       <c r="F25" s="31">
         <f>IF(F20=0,0,F14/F20)</f>
-        <v>0.1618601401472015</v>
+        <v>0.15865921441974898</v>
       </c>
       <c r="G25" s="7" t="n"/>
     </row>
@@ -7646,19 +7647,19 @@
       </c>
       <c r="C29" s="26">
         <f>Garden!C43+Garden!C44+Exchange!C47+Exchange!C48</f>
-        <v>9615.580896000001</v>
+        <v>9777.580896000001</v>
       </c>
       <c r="D29" s="26">
         <f>Garden!D43+Garden!D44+Exchange!D47+Exchange!D48</f>
-        <v>29683.731264000005</v>
+        <v>31843.731264000005</v>
       </c>
       <c r="E29" s="26">
         <f>Garden!E43+Garden!E44+Exchange!E47+Exchange!E48</f>
-        <v>70026.185088</v>
+        <v>72996.185088</v>
       </c>
       <c r="F29" s="26">
         <f>Garden!F43+Garden!F44+Exchange!F47+Exchange!F48</f>
-        <v>136476.888384</v>
+        <v>140796.888384</v>
       </c>
       <c r="G29" s="7" t="n"/>
     </row>
@@ -7870,19 +7871,19 @@
       </c>
       <c r="C37" s="28">
         <f>SUM(C28:C36)</f>
-        <v>239815.580896</v>
+        <v>239977.580896</v>
       </c>
       <c r="D37" s="28">
         <f>SUM(D28:D36)</f>
-        <v>477043.731264</v>
+        <v>479203.731264</v>
       </c>
       <c r="E37" s="28">
         <f>SUM(E28:E36)</f>
-        <v>874586.185088</v>
+        <v>877556.185088</v>
       </c>
       <c r="F37" s="28">
         <f>SUM(F28:F36)</f>
-        <v>1282276.888384</v>
+        <v>1286596.888384</v>
       </c>
       <c r="G37" s="7" t="n"/>
     </row>
@@ -7920,19 +7921,19 @@
       </c>
       <c r="C40" s="28">
         <f>C14-C37</f>
-        <v>-108252.06409600002</v>
+        <v>-106614.06409600002</v>
       </c>
       <c r="D40" s="28">
         <f>D14-D37</f>
-        <v>-115554.899264</v>
+        <v>-93714.899264</v>
       </c>
       <c r="E40" s="28">
         <f>E14-E37</f>
-        <v>-97378.39308800001</v>
+        <v>-67348.39308800001</v>
       </c>
       <c r="F40" s="28">
         <f>F14-F37</f>
-        <v>141499.52761600004</v>
+        <v>185179.52761600004</v>
       </c>
       <c r="G40" s="7" t="n"/>
     </row>
@@ -7948,19 +7949,19 @@
       </c>
       <c r="C41" s="32">
         <f>B41+C40</f>
-        <v>-126505.932234</v>
+        <v>-124867.932234</v>
       </c>
       <c r="D41" s="32">
         <f>C41+D40</f>
-        <v>-242060.831498</v>
+        <v>-218582.831498</v>
       </c>
       <c r="E41" s="32">
         <f>D41+E40</f>
-        <v>-339439.224586</v>
+        <v>-285931.224586</v>
       </c>
       <c r="F41" s="32">
         <f>E41+F40</f>
-        <v>-197939.69697</v>
+        <v>-100751.69696999999</v>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
@@ -7976,7 +7977,7 @@
       </c>
       <c r="B42" s="28">
         <f>-MIN(0,MIN(B41:F41))</f>
-        <v>339439.224586</v>
+        <v>285931.224586</v>
       </c>
       <c r="C42" s="28" t="inlineStr"/>
       <c r="D42" s="28" t="inlineStr"/>
@@ -8028,19 +8029,19 @@
       </c>
       <c r="C44" s="27">
         <f>C14/(1+Inputs!$D$128)</f>
-        <v>65781.75839999999</v>
+        <v>66681.75839999999</v>
       </c>
       <c r="D44" s="27">
         <f>D14/(1+Inputs!$E$128)</f>
-        <v>120496.27733333333</v>
+        <v>128496.27733333333</v>
       </c>
       <c r="E44" s="27">
         <f>E14/(1+Inputs!$F$128)</f>
-        <v>155441.5584</v>
+        <v>162041.5584</v>
       </c>
       <c r="F44" s="27">
         <f>F14/(1+Inputs!$G$128)</f>
-        <v>203396.63085714285</v>
+        <v>210253.77371428572</v>
       </c>
       <c r="G44" s="7" t="n"/>
     </row>
@@ -8087,7 +8088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -8294,165 +8295,167 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Three-year members incl. schools, churches and other organizations: low (founder estimate)</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Founder estimate 2026-09-30, NOT sourced. Individuals alone benchmark to about 1,000 (market-sizing.md); the rest is seats bought by schools and organizations. Source a count of San Diego schools, universities and organizations to firm this up</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Three-year members incl. schools, churches and other organizations: high (founder estimate)</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Founder estimate 2026-09-30, NOT sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>The ladder</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>TAM — US working creatives + church-based creatives</t>
         </is>
       </c>
-      <c r="B18" s="29">
+      <c r="B20" s="29">
         <f>B11+B13</f>
         <v>4750000</v>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>people who could hold a seat</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>SAM — San Diego creatives + church creatives + mapped networks, less overlap</t>
         </is>
       </c>
-      <c r="B19" s="29">
+      <c r="B21" s="29">
         <f>(B7+B9+B14)*(1-B15)</f>
         <v>35280.0</v>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>reachable in three years through partners we already know; research range 26,000–45,000 (market-sizing.md §6)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Penetration of SAM</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Paying members</t>
         </is>
-      </c>
-      <c r="C20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="B21" s="33">
-        <f>A21*B19</f>
-        <v>352.8</v>
-      </c>
-      <c r="C21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="B22" s="33">
-        <f>A22*B19</f>
-        <v>705.6</v>
       </c>
       <c r="C22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="13" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="B23" s="33">
-        <f>A23*B19</f>
-        <v>1058.3999999999999</v>
+        <f>A23*B21</f>
+        <v>352.8</v>
       </c>
       <c r="C23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="B24" s="33">
-        <f>A24*B19</f>
-        <v>1764.0</v>
+        <f>A24*B21</f>
+        <v>705.6</v>
       </c>
       <c r="C24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="B25" s="33">
+        <f>A25*B21</f>
+        <v>1058.3999999999999</v>
+      </c>
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B26" s="33">
+        <f>A26*B21</f>
+        <v>1764.0</v>
+      </c>
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="B25" s="33">
-        <f>A25*B19</f>
+      <c r="B27" s="33">
+        <f>A27*B21</f>
         <v>3528.0</v>
       </c>
-      <c r="C25" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>What the active scenario assumes</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="10" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>Paying and covered members, Y3 (Combined)</t>
-        </is>
-      </c>
-      <c r="B28" s="29">
-        <f>Combined!D21</f>
-        <v>4500</v>
-      </c>
-      <c r="C28" s="8" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  as a share of SAM</t>
-        </is>
-      </c>
-      <c r="B29" s="31">
-        <f>B28/B19</f>
-        <v>0.12755102040816327</v>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Hope*Writers alone holds ~3,200 paying members; 2–3% of SAM by Y3 is the Base case</t>
-        </is>
-      </c>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Paying and covered members, Y5 (Combined)</t>
+          <t>Paying and covered members, Y3 (Combined)</t>
         </is>
       </c>
       <c r="B30" s="29">
-        <f>Combined!F21</f>
-        <v>19000</v>
+        <f>Combined!D21</f>
+        <v>5700</v>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
     </row>
@@ -8463,38 +8466,82 @@
         </is>
       </c>
       <c r="B31" s="31">
-        <f>B30/B19</f>
-        <v>0.5385487528344671</v>
-      </c>
-      <c r="C31" s="8" t="inlineStr"/>
+        <f>B30/B21</f>
+        <v>0.16156462585034015</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Hope*Writers alone holds ~3,200 paying members; 2–3% of SAM by Y3 is the Base case</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
+          <t>Paying and covered members, Y5 (Combined)</t>
+        </is>
+      </c>
+      <c r="B32" s="29">
+        <f>Combined!F21</f>
+        <v>21000</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  as a share of SAM</t>
+        </is>
+      </c>
+      <c r="B33" s="31">
+        <f>B32/B21</f>
+        <v>0.5952380952380952</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
           <t>Garden members Y3 as a share of San Diego creatives + church creatives</t>
         </is>
       </c>
-      <c r="B32" s="31">
+      <c r="B34" s="31">
         <f>(Garden!D6+Garden!D7)/(B7+B9)</f>
         <v>0.043333333333333335</v>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>the local sanity check</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Active scenario Y3 members vs the founder-estimated range (5,000 to 10,000)</t>
+        </is>
+      </c>
+      <c r="B35" s="34" t="str">
+        <f>IF(Combined!D21&lt;B16,"below",IF(Combined!D21&gt;B17,"above","inside"))</f>
+        <v>inside</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Base should sit inside the range; Conservative below it (individuals only); Fundable at or above the top</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Paying and covered members, Y5, as a share of US TAM</t>
         </is>
       </c>
-      <c r="B33" s="31">
-        <f>Combined!F21/B18</f>
-        <v>0.004</v>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="B36" s="31">
+        <f>Combined!F21/B20</f>
+        <v>0.004421052631578947</v>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>the national sanity check: partner communities and org seats are not confined to San Diego from Y2 on</t>
         </is>
@@ -8570,7 +8617,7 @@
       </c>
       <c r="B4" s="24">
         <f>Combined!D21</f>
-        <v>4500</v>
+        <v>5700</v>
       </c>
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="7" t="n"/>
@@ -8585,9 +8632,9 @@
           <t>Active scenario Y3 revenue per member</t>
         </is>
       </c>
-      <c r="B5" s="34">
+      <c r="B5" s="35">
         <f>Combined!D24</f>
-        <v>80.33085155555555</v>
+        <v>67.6296196491228</v>
       </c>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
@@ -8604,7 +8651,7 @@
       </c>
       <c r="B6" s="26">
         <f>Combined!D37</f>
-        <v>477043.731264</v>
+        <v>479203.731264</v>
       </c>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="7" t="n"/>
@@ -8629,25 +8676,25 @@
           <t>Members \ $ per member</t>
         </is>
       </c>
-      <c r="B8" s="35" t="n">
+      <c r="B8" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="C8" s="35" t="n">
+      <c r="C8" s="36" t="n">
         <v>40</v>
       </c>
-      <c r="D8" s="35" t="n">
+      <c r="D8" s="36" t="n">
         <v>60</v>
       </c>
-      <c r="E8" s="35" t="n">
+      <c r="E8" s="36" t="n">
         <v>90</v>
       </c>
-      <c r="F8" s="35" t="n">
+      <c r="F8" s="36" t="n">
         <v>120</v>
       </c>
-      <c r="G8" s="35" t="n">
+      <c r="G8" s="36" t="n">
         <v>160</v>
       </c>
-      <c r="H8" s="35" t="n">
+      <c r="H8" s="36" t="n">
         <v>200</v>
       </c>
     </row>
@@ -8655,31 +8702,31 @@
       <c r="A9" s="18" t="n">
         <v>1000</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B9" s="37">
         <f>$A9*B$8</f>
         <v>20000</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="37">
         <f>$A9*C$8</f>
         <v>40000</v>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="37">
         <f>$A9*D$8</f>
         <v>60000</v>
       </c>
-      <c r="E9" s="36">
+      <c r="E9" s="37">
         <f>$A9*E$8</f>
         <v>90000</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="37">
         <f>$A9*F$8</f>
         <v>120000</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <f>$A9*G$8</f>
         <v>160000</v>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="37">
         <f>$A9*H$8</f>
         <v>200000</v>
       </c>
@@ -8688,31 +8735,31 @@
       <c r="A10" s="18" t="n">
         <v>2500</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="37">
         <f>$A10*B$8</f>
         <v>50000</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="37">
         <f>$A10*C$8</f>
         <v>100000</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="37">
         <f>$A10*D$8</f>
         <v>150000</v>
       </c>
-      <c r="E10" s="36">
+      <c r="E10" s="37">
         <f>$A10*E$8</f>
         <v>225000</v>
       </c>
-      <c r="F10" s="36">
+      <c r="F10" s="37">
         <f>$A10*F$8</f>
         <v>300000</v>
       </c>
-      <c r="G10" s="36">
+      <c r="G10" s="37">
         <f>$A10*G$8</f>
         <v>400000</v>
       </c>
-      <c r="H10" s="36">
+      <c r="H10" s="37">
         <f>$A10*H$8</f>
         <v>500000</v>
       </c>
@@ -8721,31 +8768,31 @@
       <c r="A11" s="18" t="n">
         <v>5000</v>
       </c>
-      <c r="B11" s="36">
+      <c r="B11" s="37">
         <f>$A11*B$8</f>
         <v>100000</v>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="37">
         <f>$A11*C$8</f>
         <v>200000</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="37">
         <f>$A11*D$8</f>
         <v>300000</v>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="37">
         <f>$A11*E$8</f>
         <v>450000</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="37">
         <f>$A11*F$8</f>
         <v>600000</v>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="37">
         <f>$A11*G$8</f>
         <v>800000</v>
       </c>
-      <c r="H11" s="36">
+      <c r="H11" s="37">
         <f>$A11*H$8</f>
         <v>1000000</v>
       </c>
@@ -8754,31 +8801,31 @@
       <c r="A12" s="18" t="n">
         <v>10000</v>
       </c>
-      <c r="B12" s="36">
+      <c r="B12" s="37">
         <f>$A12*B$8</f>
         <v>200000</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="37">
         <f>$A12*C$8</f>
         <v>400000</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="37">
         <f>$A12*D$8</f>
         <v>600000</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="37">
         <f>$A12*E$8</f>
         <v>900000</v>
       </c>
-      <c r="F12" s="36">
+      <c r="F12" s="37">
         <f>$A12*F$8</f>
         <v>1200000</v>
       </c>
-      <c r="G12" s="36">
+      <c r="G12" s="37">
         <f>$A12*G$8</f>
         <v>1600000</v>
       </c>
-      <c r="H12" s="36">
+      <c r="H12" s="37">
         <f>$A12*H$8</f>
         <v>2000000</v>
       </c>
@@ -8787,31 +8834,31 @@
       <c r="A13" s="18" t="n">
         <v>20000</v>
       </c>
-      <c r="B13" s="36">
+      <c r="B13" s="37">
         <f>$A13*B$8</f>
         <v>400000</v>
       </c>
-      <c r="C13" s="36">
+      <c r="C13" s="37">
         <f>$A13*C$8</f>
         <v>800000</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="37">
         <f>$A13*D$8</f>
         <v>1200000</v>
       </c>
-      <c r="E13" s="36">
+      <c r="E13" s="37">
         <f>$A13*E$8</f>
         <v>1800000</v>
       </c>
-      <c r="F13" s="36">
+      <c r="F13" s="37">
         <f>$A13*F$8</f>
         <v>2400000</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="37">
         <f>$A13*G$8</f>
         <v>3200000</v>
       </c>
-      <c r="H13" s="36">
+      <c r="H13" s="37">
         <f>$A13*H$8</f>
         <v>4000000</v>
       </c>
@@ -8820,31 +8867,31 @@
       <c r="A14" s="18" t="n">
         <v>40000</v>
       </c>
-      <c r="B14" s="36">
+      <c r="B14" s="37">
         <f>$A14*B$8</f>
         <v>800000</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="37">
         <f>$A14*C$8</f>
         <v>1600000</v>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="37">
         <f>$A14*D$8</f>
         <v>2400000</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="37">
         <f>$A14*E$8</f>
         <v>3600000</v>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="37">
         <f>$A14*F$8</f>
         <v>4800000</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="37">
         <f>$A14*G$8</f>
         <v>6400000</v>
       </c>
-      <c r="H14" s="36">
+      <c r="H14" s="37">
         <f>$A14*H$8</f>
         <v>8000000</v>
       </c>

</xml_diff>

<commit_message>
Model README: refresh results, targets and formula count; add metro note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETG5M27XfcTD2TyhhuebtG
</commit_message>
<xml_diff>
--- a/docs/financial-model-5yr-v2.xlsx
+++ b/docs/financial-model-5yr-v2.xlsx
@@ -634,7 +634,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>4. Results (cost side rebuilt 2026-09-30: budget by function, founders full time before any employee, founder pay starting when there is money for it and ramping, payroll load applied). Revenue is unchanged: Base $36k / $133k / $385k / $810k / $1.47M. The Base and Fundable cost, EBITDA and cash figures are on the Combined sheet; the README of the docs folder and docs/funding/cfo-memo-ask-and-spend.md carry the discussion.</t>
+          <t>4. Results (2026-09-30: franchise metros as explicit drivers, a Base team of four, founder pay inside the functions). Base revenue $36k / $146k / $461k / $1.06M / $2.11M; EBITDA -$192k / -$313k / -$318k / -$3k / +$672k, so breakeven in year four and about $826k of cumulative capital at the low point. Fundable revenue $80k / $363k / $1.38M / $3.89M / $9.29M with 40 metros and a team of 18, EBITDA positive in year four. Conservative: $17k growing to $313k with 5 metros, not profitable in five years. Costs, EBITDA and cash are on the Combined sheet; docs/funding/cfo-memo-ask-and-spend.md carries the discussion.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>4c. Founder targets (2026-09-30): at least 3,000 paying INDIVIDUALS by year three, and 5,000-10,000 members once organizations buy seats for their stakeholders. Base meets both (about 3,200 individuals and 5,700 members in Y3); Conservative does not (about 950 individuals). Organization-bought seats are about 20% of Y3 revenue. Neither target is sourced yet.</t>
+          <t>4c. Founder targets (2026-09-30): at least 3,000 paying INDIVIDUALS by year three, and 5,000-10,000 members once organizations buy seats for their stakeholders. Base meets both (about 5,100 individuals and 7,600 members in Y3, with 6 franchise metros live); Conservative does not (about 1,250 individuals and 1,570 members). Organization-bought seats are about 17% of Y3 Base revenue. Neither target is sourced yet.</t>
         </is>
       </c>
     </row>
@@ -660,12 +660,16 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>4d. Franchise metros (Exchange sheet, rows 16 to 19; every number is a variable): new metros launched per year (cumulative by Y5: Conservative 5, Base 20, Fundable 40), cost to launch a metro ($8k / $12k / $20k, one time), cost to support an active metro ($4k / $6k / $10k a year) and partner communities per active metro (Base: 2 in the launch year rising to 6). A metro costs relationships and some marketing, not staff.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>VALUES: this file was built with openpyxl and its formulas were evaluated with a Python formula engine (pycel; 1,009 formulas, 0 errors in every scenario) because LibreOffice is not available in the build sandbox. Excel and Google Sheets recalculate every formula on open, so what you see is live.</t>
+          <t>VALUES: this file was built with openpyxl and its formulas were evaluated with a Python formula engine (pycel; 1,138 formulas, 0 errors in every scenario) because LibreOffice is not available in the build sandbox. Excel and Google Sheets recalculate every formula on open, so what you see is live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Base case: three metros by month 18, six by end of year two; three founders on the team slide
Model: Base metro launches 0/6/3/5/6 (nine metros and San Diego is ten
cities by year three). Base revenue $36k/$172k/$499k/$1.11M/$2.11M,
breakeven in year four, capital low point $851k in year three. 18-month
window: spend $497k, revenue $122k, net need $374k, so $350k is 17
months of runway. Deck use of funds (75% on community and GTM), ask,
impact, market, business and team slides, CFO memo, fresh-look memo and
README updated. Team slide shows three founders; Patricia Sinay is
Chief Creative & Programs.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETG5M27XfcTD2TyhhuebtG
</commit_message>
<xml_diff>
--- a/docs/financial-model-5yr-v2.xlsx
+++ b/docs/financial-model-5yr-v2.xlsx
@@ -634,7 +634,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>4. Results (2026-09-30: franchise metros as explicit drivers, a Base team of four, founder pay inside the functions). Base revenue $36k / $146k / $461k / $1.06M / $2.11M; EBITDA -$192k / -$313k / -$318k / -$3k / +$672k, so breakeven in year four and about $826k of cumulative capital at the low point. Fundable revenue $80k / $363k / $1.38M / $3.89M / $9.29M with 40 metros and a team of 18, EBITDA positive in year four. Conservative: $17k growing to $313k with 5 metros, not profitable in five years. Costs, EBITDA and cash are on the Combined sheet; docs/funding/cfo-memo-ask-and-spend.md carries the discussion.</t>
+          <t>4. Results (2026-10-01: metros as explicit drivers, a Base team of four, founder pay inside the functions). Base revenue $36k / $172k / $499k / $1.11M / $2.11M; EBITDA -$192k / -$365k / -$294k / +$30k / +$696k, so breakeven in year four and about $851k of cumulative capital at the low point, in year three. Fundable revenue $80k / $363k / $1.38M / $3.89M / $9.29M with 40 metros and a team of 18, EBITDA positive in year four. Conservative: $17k growing to $313k with 5 metros, not profitable in five years. Costs, EBITDA and cash are on the Combined sheet; docs/funding/cfo-memo-ask-and-spend.md carries the discussion.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>4c. Founder targets (2026-09-30): at least 3,000 paying INDIVIDUALS by year three, and 5,000-10,000 members once organizations buy seats for their stakeholders. Base meets both (about 5,100 individuals and 7,600 members in Y3, with 6 franchise metros live); Conservative does not (about 1,250 individuals and 1,570 members). Organization-bought seats are about 17% of Y3 Base revenue. Neither target is sourced yet.</t>
+          <t>4c. Founder targets (2026-09-30): at least 3,000 paying INDIVIDUALS by year three, and 5,000-10,000 members once organizations buy seats for their stakeholders. Base meets both (about 6,100 individuals and 8,600 members in Y3, with 9 metros live); Conservative does not (about 1,250 individuals and 1,570 members). Organization-bought seats are about 15% of Y3 Base revenue. Neither target is sourced yet.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>4d. Franchise metros (Exchange sheet, rows 16 to 19; every number is a variable): new metros launched per year (cumulative by Y5: Conservative 5, Base 20, Fundable 40), cost to launch a metro ($8k / $12k / $20k, one time), cost to support an active metro ($4k / $6k / $10k a year) and partner communities per active metro (Base: 2 in the launch year rising to 6). A metro costs relationships and some marketing, not staff.</t>
+          <t>4d. Metros (Exchange sheet, rows 16 to 19; every number is a variable): new metros launched per year (Base 0 / 6 / 3 / 5 / 6: three by month 18, six by the end of year two, nine by the end of year three, ten cities with San Diego; cumulative by Y5 Conservative 5, Base 20, Fundable 40), cost to launch a metro ($8k / $12k / $20k, one time), cost to support an active metro ($4k / $6k / $10k a year) and partner communities per active metro (Base: 2 in the launch year rising to 6). A metro costs relationships and some marketing, not staff.</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="H130" s="8" t="inlineStr">
         <is>
-          <t>A metro is a cluster of communities led by their own people on our infrastructure (Nashville, Las Vegas, Los Angeles, Austin, Atlanta, Dallas-Fort Worth, Phoenix, Denver, Seattle first). Cumulative by Y5: Conservative 5, Base 20, Fundable 40</t>
+          <t>A metro is a cluster of communities led by their own people on our infrastructure (Nashville, Las Vegas, Los Angeles, Austin, Atlanta, Dallas-Fort Worth, Phoenix, Denver, Seattle first). Cumulative by Y5: Conservative 5, Base 20, Fundable 40. Base: 3 launched by month 18, 6 by the end of year two, 9 by the end of year three (San Diego plus nine metros is ten cities)</t>
         </is>
       </c>
     </row>
@@ -3642,16 +3642,16 @@
         <v>0</v>
       </c>
       <c r="D131" s="18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E131" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F131" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G131" s="18" t="n">
         <v>6</v>
-      </c>
-      <c r="G131" s="18" t="n">
-        <v>8</v>
       </c>
       <c r="H131" s="7" t="n"/>
     </row>
@@ -3692,19 +3692,19 @@
       </c>
       <c r="D133" s="19">
         <f>CHOOSE(Inputs!$B$29,D130,D131,D132)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E133" s="19">
         <f>CHOOSE(Inputs!$B$29,E130,E131,E132)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F133" s="19">
         <f>CHOOSE(Inputs!$B$29,F130,F131,F132)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G133" s="19">
         <f>CHOOSE(Inputs!$B$29,G130,G131,G132)</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H133" s="7" t="n"/>
     </row>
@@ -8532,19 +8532,19 @@
       </c>
       <c r="C16" s="24">
         <f>Inputs!$D$133</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D16" s="24">
         <f>Inputs!$E$133</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" s="24">
         <f>Inputs!$F$133</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" s="24">
         <f>Inputs!$G$133</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G16" s="7" t="n"/>
     </row>
@@ -8644,15 +8644,15 @@
       </c>
       <c r="C20" s="29">
         <f>B20+C16</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D20" s="29">
         <f>C20+D16</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E20" s="29">
         <f>D20+E16</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F20" s="29">
         <f>E20+F16</f>
@@ -8676,15 +8676,15 @@
       </c>
       <c r="C21" s="29">
         <f>C20*C19</f>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D21" s="29">
         <f>D20*D19</f>
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E21" s="29">
         <f>E20*E19</f>
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F21" s="29">
         <f>F20*F19</f>
@@ -8708,15 +8708,15 @@
       </c>
       <c r="C22" s="31">
         <f>C6+C21</f>
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D22" s="31">
         <f>D6+D21</f>
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E22" s="31">
         <f>E6+E21</f>
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F22" s="31">
         <f>F6+F21</f>
@@ -8736,15 +8736,15 @@
       </c>
       <c r="C23" s="29">
         <f>C22*C7</f>
-        <v>1080</v>
+        <v>1800</v>
       </c>
       <c r="D23" s="29">
         <f>D22*D7</f>
-        <v>4320</v>
+        <v>5280</v>
       </c>
       <c r="E23" s="29">
         <f>E22*E7</f>
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="F23" s="29">
         <f>F22*F7</f>
@@ -8790,15 +8790,15 @@
       </c>
       <c r="C26" s="27">
         <f>C23*12*Inputs!$B$5*(1-Inputs!$B$7*(1-Inputs!$B$21))</f>
-        <v>120958.27200000001</v>
+        <v>201597.12</v>
       </c>
       <c r="D26" s="27">
         <f>D23*12*Inputs!$B$5*(1-Inputs!$B$7*(1-Inputs!$B$21))</f>
-        <v>483833.08800000005</v>
+        <v>591351.552</v>
       </c>
       <c r="E26" s="27">
         <f>E23*12*Inputs!$B$5*(1-Inputs!$B$7*(1-Inputs!$B$21))</f>
-        <v>1343980.8</v>
+        <v>1455979.2</v>
       </c>
       <c r="F26" s="27">
         <f>F23*12*Inputs!$B$5*(1-Inputs!$B$7*(1-Inputs!$B$21))</f>
@@ -8850,15 +8850,15 @@
       </c>
       <c r="C28" s="27">
         <f>(C23+C8)*C10</f>
-        <v>110400</v>
+        <v>168000</v>
       </c>
       <c r="D28" s="27">
         <f>(D23+D8)*D10</f>
-        <v>632000</v>
+        <v>728000</v>
       </c>
       <c r="E28" s="27">
         <f>(E23+E8)*E10</f>
-        <v>1860000</v>
+        <v>1980000</v>
       </c>
       <c r="F28" s="27">
         <f>(F23+F8)*F10</f>
@@ -8878,15 +8878,15 @@
       </c>
       <c r="C29" s="27">
         <f>C22*C9</f>
-        <v>144000</v>
+        <v>240000</v>
       </c>
       <c r="D29" s="27">
         <f>D22*D9</f>
-        <v>648000</v>
+        <v>792000</v>
       </c>
       <c r="E29" s="27">
         <f>E22*E9</f>
-        <v>1920000</v>
+        <v>2080000</v>
       </c>
       <c r="F29" s="27">
         <f>F22*F9</f>
@@ -8990,15 +8990,15 @@
       </c>
       <c r="C33" s="27">
         <f>C22*C11*Inputs!$B$15*12</f>
-        <v>3780</v>
+        <v>6300</v>
       </c>
       <c r="D33" s="27">
         <f>D22*D11*Inputs!$B$15*12</f>
-        <v>14580</v>
+        <v>17820</v>
       </c>
       <c r="E33" s="27">
         <f>E22*E11*Inputs!$B$15*12</f>
-        <v>36000</v>
+        <v>39000</v>
       </c>
       <c r="F33" s="27">
         <f>F22*F11*Inputs!$B$15*12</f>
@@ -9046,15 +9046,15 @@
       </c>
       <c r="C35" s="28">
         <f>SUM(C26:C34)</f>
-        <v>478098.272</v>
+        <v>714857.12</v>
       </c>
       <c r="D35" s="28">
         <f>SUM(D26:D34)</f>
-        <v>2185293.088</v>
+        <v>2536051.552</v>
       </c>
       <c r="E35" s="28">
         <f>SUM(E26:E34)</f>
-        <v>6012180.8</v>
+        <v>6407179.2</v>
       </c>
       <c r="F35" s="28">
         <f>SUM(F26:F34)</f>
@@ -9096,15 +9096,15 @@
       </c>
       <c r="C38" s="27">
         <f>(C26+C27)*Inputs!$B$10</f>
-        <v>15095.8272</v>
+        <v>23159.712</v>
       </c>
       <c r="D38" s="27">
         <f>(D26+D27)*Inputs!$B$10</f>
-        <v>68383.3088</v>
+        <v>79135.15520000001</v>
       </c>
       <c r="E38" s="27">
         <f>(E26+E27)*Inputs!$B$10</f>
-        <v>169398.08000000002</v>
+        <v>180597.92</v>
       </c>
       <c r="F38" s="27">
         <f>(F26+F27)*Inputs!$B$10</f>
@@ -9124,15 +9124,15 @@
       </c>
       <c r="C39" s="27">
         <f>C28*Inputs!$B$11</f>
-        <v>11040.0</v>
+        <v>16800.0</v>
       </c>
       <c r="D39" s="27">
         <f>D28*Inputs!$B$11</f>
-        <v>63200.0</v>
+        <v>72800.0</v>
       </c>
       <c r="E39" s="27">
         <f>E28*Inputs!$B$11</f>
-        <v>186000.0</v>
+        <v>198000.0</v>
       </c>
       <c r="F39" s="27">
         <f>F28*Inputs!$B$11</f>
@@ -9152,15 +9152,15 @@
       </c>
       <c r="C40" s="27">
         <f>C29*Inputs!$B$12</f>
-        <v>14400.0</v>
+        <v>24000.0</v>
       </c>
       <c r="D40" s="27">
         <f>D29*Inputs!$B$12</f>
-        <v>64800.0</v>
+        <v>79200.0</v>
       </c>
       <c r="E40" s="27">
         <f>E29*Inputs!$B$12</f>
-        <v>192000.0</v>
+        <v>208000.0</v>
       </c>
       <c r="F40" s="27">
         <f>F29*Inputs!$B$12</f>
@@ -9264,15 +9264,15 @@
       </c>
       <c r="C44" s="27">
         <f>C33</f>
-        <v>3780</v>
+        <v>6300</v>
       </c>
       <c r="D44" s="27">
         <f>D33</f>
-        <v>14580</v>
+        <v>17820</v>
       </c>
       <c r="E44" s="27">
         <f>E33</f>
-        <v>36000</v>
+        <v>39000</v>
       </c>
       <c r="F44" s="27">
         <f>F33</f>
@@ -9320,15 +9320,15 @@
       </c>
       <c r="C46" s="28">
         <f>SUM(C38:C45)</f>
-        <v>75275.8272</v>
+        <v>101219.712</v>
       </c>
       <c r="D46" s="28">
         <f>SUM(D38:D45)</f>
-        <v>303843.3088</v>
+        <v>341835.15520000004</v>
       </c>
       <c r="E46" s="28">
         <f>SUM(E38:E45)</f>
-        <v>800598.0800000001</v>
+        <v>842797.92</v>
       </c>
       <c r="F46" s="28">
         <f>SUM(F38:F45)</f>
@@ -9370,15 +9370,15 @@
       </c>
       <c r="C49" s="27">
         <f>(C26+C27)*(1-Inputs!$B$10)</f>
-        <v>135862.4448</v>
+        <v>208437.408</v>
       </c>
       <c r="D49" s="27">
         <f>(D26+D27)*(1-Inputs!$B$10)</f>
-        <v>615449.7792</v>
+        <v>712216.3968</v>
       </c>
       <c r="E49" s="27">
         <f>(E26+E27)*(1-Inputs!$B$10)</f>
-        <v>1524582.72</v>
+        <v>1625381.28</v>
       </c>
       <c r="F49" s="27">
         <f>(F26+F27)*(1-Inputs!$B$10)</f>
@@ -9398,15 +9398,15 @@
       </c>
       <c r="C50" s="27">
         <f>C28*(1-Inputs!$B$11)+C29*(1-Inputs!$B$12)</f>
-        <v>228960</v>
+        <v>367200</v>
       </c>
       <c r="D50" s="27">
         <f>D28*(1-Inputs!$B$11)+D29*(1-Inputs!$B$12)</f>
-        <v>1152000</v>
+        <v>1368000</v>
       </c>
       <c r="E50" s="27">
         <f>E28*(1-Inputs!$B$11)+E29*(1-Inputs!$B$12)</f>
-        <v>3402000</v>
+        <v>3654000</v>
       </c>
       <c r="F50" s="27">
         <f>F28*(1-Inputs!$B$11)+F29*(1-Inputs!$B$12)</f>
@@ -9476,15 +9476,15 @@
       </c>
       <c r="C54" s="27">
         <f>C26*Inputs!$B$21*(Inputs!$B$19+Inputs!$B$20/Inputs!$B$5)+C26*(1-Inputs!$B$21)*Inputs!$B$19</f>
-        <v>5685.038783999999</v>
+        <v>9475.06464</v>
       </c>
       <c r="D54" s="27">
         <f>D26*Inputs!$B$21*(Inputs!$B$19+Inputs!$B$20/Inputs!$B$5)+D26*(1-Inputs!$B$21)*Inputs!$B$19</f>
-        <v>22740.155135999998</v>
+        <v>27793.522944</v>
       </c>
       <c r="E54" s="27">
         <f>E26*Inputs!$B$21*(Inputs!$B$19+Inputs!$B$20/Inputs!$B$5)+E26*(1-Inputs!$B$21)*Inputs!$B$19</f>
-        <v>63167.0976</v>
+        <v>68431.02239999999</v>
       </c>
       <c r="F54" s="27">
         <f>F26*Inputs!$B$21*(Inputs!$B$19+Inputs!$B$20/Inputs!$B$5)+F26*(1-Inputs!$B$21)*Inputs!$B$19</f>
@@ -9504,15 +9504,15 @@
       </c>
       <c r="C55" s="27">
         <f>(C49+C50)*Inputs!$B$22</f>
-        <v>3648.224448</v>
+        <v>5756.3740800000005</v>
       </c>
       <c r="D55" s="27">
         <f>(D49+D50)*Inputs!$B$22</f>
-        <v>17674.497792000002</v>
+        <v>20802.163968</v>
       </c>
       <c r="E55" s="27">
         <f>(E49+E50)*Inputs!$B$22</f>
-        <v>49265.8272</v>
+        <v>52793.81280000001</v>
       </c>
       <c r="F55" s="27">
         <f>(F49+F50)*Inputs!$B$22</f>
@@ -9532,15 +9532,15 @@
       </c>
       <c r="C56" s="28">
         <f>C46-C54-C55</f>
-        <v>65942.563968</v>
+        <v>85988.27328000001</v>
       </c>
       <c r="D56" s="28">
         <f>D46-D54-D55</f>
-        <v>263428.655872</v>
+        <v>293239.46828800003</v>
       </c>
       <c r="E56" s="28">
         <f>E46-E54-E55</f>
-        <v>688165.1552000002</v>
+        <v>721573.0848000001</v>
       </c>
       <c r="F56" s="28">
         <f>F46-F54-F55</f>
@@ -9569,15 +9569,15 @@
       </c>
       <c r="C58" s="30">
         <f>IF((C23+C8)=0,0,C46/(C23+C8))</f>
-        <v>54.54770086956522</v>
+        <v>48.199862857142854</v>
       </c>
       <c r="D58" s="30">
         <f>IF((D23+D8)=0,0,D46/(D23+D8))</f>
-        <v>48.07647291139241</v>
+        <v>46.955378461538466</v>
       </c>
       <c r="E58" s="30">
         <f>IF((E23+E8)=0,0,E46/(E23+E8))</f>
-        <v>51.65148903225807</v>
+        <v>51.07866181818182</v>
       </c>
       <c r="F58" s="30">
         <f>IF((F23+F8)=0,0,F46/(F23+F8))</f>
@@ -9597,15 +9597,15 @@
       </c>
       <c r="C59" s="27">
         <f>IF(C6=0,0,C46/C6)</f>
-        <v>6272.9856</v>
+        <v>8434.976</v>
       </c>
       <c r="D59" s="27">
         <f>IF(D6=0,0,D46/D6)</f>
-        <v>10128.110293333333</v>
+        <v>11394.505173333335</v>
       </c>
       <c r="E59" s="27">
         <f>IF(E6=0,0,E46/E6)</f>
-        <v>13343.301333333335</v>
+        <v>14046.632000000001</v>
       </c>
       <c r="F59" s="27">
         <f>IF(F6=0,0,F46/F6)</f>
@@ -9732,15 +9732,15 @@
       </c>
       <c r="C6" s="26">
         <f>Garden!C27+Exchange!C38</f>
-        <v>50855.4592</v>
+        <v>58919.344</v>
       </c>
       <c r="D6" s="26">
         <f>Garden!D27+Exchange!D38</f>
-        <v>148262.5248</v>
+        <v>159014.3712</v>
       </c>
       <c r="E6" s="26">
         <f>Garden!E27+Exchange!E38</f>
-        <v>301756.83200000005</v>
+        <v>312956.672</v>
       </c>
       <c r="F6" s="26">
         <f>Garden!F27+Exchange!F38</f>
@@ -9760,15 +9760,15 @@
       </c>
       <c r="C7" s="26">
         <f>Garden!C28+Exchange!C39</f>
-        <v>17040</v>
+        <v>22800</v>
       </c>
       <c r="D7" s="26">
         <f>Garden!D28+Exchange!D39</f>
-        <v>79450</v>
+        <v>89050</v>
       </c>
       <c r="E7" s="26">
         <f>Garden!E28+Exchange!E39</f>
-        <v>217500</v>
+        <v>229500</v>
       </c>
       <c r="F7" s="26">
         <f>Garden!F28+Exchange!F39</f>
@@ -9788,15 +9788,15 @@
       </c>
       <c r="C8" s="26">
         <f>Garden!C29+Exchange!C40</f>
-        <v>19200</v>
+        <v>28800</v>
       </c>
       <c r="D8" s="26">
         <f>Garden!D29+Exchange!D40</f>
-        <v>77800</v>
+        <v>92200</v>
       </c>
       <c r="E8" s="26">
         <f>Garden!E29+Exchange!E40</f>
-        <v>217200</v>
+        <v>233200</v>
       </c>
       <c r="F8" s="26">
         <f>Garden!F29+Exchange!F40</f>
@@ -9900,15 +9900,15 @@
       </c>
       <c r="C12" s="26">
         <f>Exchange!C44</f>
-        <v>3780</v>
+        <v>6300</v>
       </c>
       <c r="D12" s="26">
         <f>Exchange!D44</f>
-        <v>14580</v>
+        <v>17820</v>
       </c>
       <c r="E12" s="26">
         <f>Exchange!E44</f>
-        <v>36000</v>
+        <v>39000</v>
       </c>
       <c r="F12" s="26">
         <f>Exchange!F44</f>
@@ -9956,15 +9956,15 @@
       </c>
       <c r="C14" s="28">
         <f>SUM(C6:C13)</f>
-        <v>146335.45919999998</v>
+        <v>172279.34399999998</v>
       </c>
       <c r="D14" s="28">
         <f>SUM(D6:D13)</f>
-        <v>461472.5248</v>
+        <v>499464.3712</v>
       </c>
       <c r="E14" s="28">
         <f>SUM(E6:E13)</f>
-        <v>1063406.832</v>
+        <v>1105606.672</v>
       </c>
       <c r="F14" s="28">
         <f>SUM(F6:F13)</f>
@@ -10012,15 +10012,15 @@
       </c>
       <c r="C16" s="26">
         <f>Exchange!C46</f>
-        <v>75275.8272</v>
+        <v>101219.712</v>
       </c>
       <c r="D16" s="26">
         <f>Exchange!D46</f>
-        <v>303843.3088</v>
+        <v>341835.15520000004</v>
       </c>
       <c r="E16" s="26">
         <f>Exchange!E46</f>
-        <v>800598.0800000001</v>
+        <v>842797.92</v>
       </c>
       <c r="F16" s="26">
         <f>Exchange!F46</f>
@@ -10040,15 +10040,15 @@
       </c>
       <c r="C17" s="32">
         <f>IF(C14=0,0,(C10+C12+C13)/C14)</f>
-        <v>0.17248040999757905</v>
+        <v>0.16113365279589179</v>
       </c>
       <c r="D17" s="32">
         <f>IF(D14=0,0,(D10+D12+D13)/D14)</f>
-        <v>0.16677049198834556</v>
+        <v>0.16057201399033447</v>
       </c>
       <c r="E17" s="32">
         <f>IF(E14=0,0,(E10+E12+E13)/E14)</f>
-        <v>0.17815383002918306</v>
+        <v>0.17406732871091066</v>
       </c>
       <c r="F17" s="32">
         <f>IF(F14=0,0,(F10+F12+F13)/F14)</f>
@@ -10090,15 +10090,15 @@
       </c>
       <c r="C20" s="26">
         <f>Garden!C24+Exchange!C35</f>
-        <v>767617.536</v>
+        <v>1004376.384</v>
       </c>
       <c r="D20" s="26">
         <f>Garden!D24+Exchange!D35</f>
-        <v>2847551.52</v>
+        <v>3198309.984</v>
       </c>
       <c r="E20" s="26">
         <f>Garden!E24+Exchange!E35</f>
-        <v>7178898.304</v>
+        <v>7573896.704</v>
       </c>
       <c r="F20" s="26">
         <f>Garden!F24+Exchange!F35</f>
@@ -10118,15 +10118,15 @@
       </c>
       <c r="C21" s="24">
         <f>Garden!C6+Garden!C7+Exchange!C23+Exchange!C8</f>
-        <v>1980</v>
+        <v>2700</v>
       </c>
       <c r="D21" s="24">
         <f>Garden!D6+Garden!D7+Exchange!D23+Exchange!D8</f>
-        <v>7620</v>
+        <v>8580</v>
       </c>
       <c r="E21" s="24">
         <f>Garden!E6+Garden!E7+Exchange!E23+Exchange!E8</f>
-        <v>17600</v>
+        <v>18600</v>
       </c>
       <c r="F21" s="24">
         <f>Garden!F6+Garden!F7+Exchange!F23+Exchange!F8</f>
@@ -10146,15 +10146,15 @@
       </c>
       <c r="C22" s="24">
         <f>Garden!C6+Exchange!C23</f>
-        <v>1480</v>
+        <v>2200</v>
       </c>
       <c r="D22" s="24">
         <f>Garden!D6+Exchange!D23</f>
-        <v>5120</v>
+        <v>6080</v>
       </c>
       <c r="E22" s="24">
         <f>Garden!E6+Exchange!E23</f>
-        <v>13200</v>
+        <v>14200</v>
       </c>
       <c r="F22" s="24">
         <f>Garden!F6+Exchange!F23</f>
@@ -10238,15 +10238,15 @@
       </c>
       <c r="C25" s="32">
         <f>IF(C14=0,0,C24/C14)</f>
-        <v>0.12983866045776554</v>
+        <v>0.11028600155338415</v>
       </c>
       <c r="D25" s="32">
         <f>IF(D14=0,0,D24/D14)</f>
-        <v>0.1652319388527982</v>
+        <v>0.15266354197958856</v>
       </c>
       <c r="E25" s="32">
         <f>IF(E14=0,0,E24/E14)</f>
-        <v>0.1375766974572155</v>
+        <v>0.13232554009044548</v>
       </c>
       <c r="F25" s="32">
         <f>IF(F14=0,0,F24/F14)</f>
@@ -10266,15 +10266,15 @@
       </c>
       <c r="C26" s="24">
         <f>1+Exchange!C22</f>
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D26" s="24">
         <f>1+Exchange!D22</f>
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E26" s="24">
         <f>1+Exchange!E22</f>
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="F26" s="24">
         <f>1+Exchange!F22</f>
@@ -10294,15 +10294,15 @@
       </c>
       <c r="C27" s="24">
         <f>Exchange!C20</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D27" s="24">
         <f>Exchange!D20</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E27" s="24">
         <f>Exchange!E20</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F27" s="24">
         <f>Exchange!F20</f>
@@ -10322,15 +10322,15 @@
       </c>
       <c r="C28" s="26">
         <f>Garden!C19*(1-Inputs!$B$11)+Garden!C20*(1-Inputs!$B$12)+Garden!C38+Exchange!C50+Exchange!C51</f>
-        <v>433919.632</v>
+        <v>572159.632</v>
       </c>
       <c r="D28" s="26">
         <f>Garden!D19*(1-Inputs!$B$11)+Garden!D20*(1-Inputs!$B$12)+Garden!D38+Exchange!D50+Exchange!D51</f>
-        <v>1657129.216</v>
+        <v>1873129.216</v>
       </c>
       <c r="E28" s="26">
         <f>Garden!E19*(1-Inputs!$B$11)+Garden!E20*(1-Inputs!$B$12)+Garden!E38+Exchange!E50+Exchange!E51</f>
-        <v>4359658.752</v>
+        <v>4611658.752</v>
       </c>
       <c r="F28" s="26">
         <f>Garden!F19*(1-Inputs!$B$11)+Garden!F20*(1-Inputs!$B$12)+Garden!F38+Exchange!F50+Exchange!F51</f>
@@ -10354,15 +10354,15 @@
       </c>
       <c r="C29" s="30">
         <f>IF(C21=0,0,C14/C21)</f>
-        <v>73.90679757575757</v>
+        <v>63.80716444444444</v>
       </c>
       <c r="D29" s="30">
         <f>IF(D21=0,0,D14/D21)</f>
-        <v>60.56069879265092</v>
+        <v>58.212630675990674</v>
       </c>
       <c r="E29" s="30">
         <f>IF(E21=0,0,E14/E21)</f>
-        <v>60.42084272727272</v>
+        <v>59.44121892473118</v>
       </c>
       <c r="F29" s="30">
         <f>IF(F21=0,0,F14/F21)</f>
@@ -10382,15 +10382,15 @@
       </c>
       <c r="C30" s="32">
         <f>IF(C20=0,0,C14/C20)</f>
-        <v>0.19063589917779053</v>
+        <v>0.17152866867885255</v>
       </c>
       <c r="D30" s="32">
         <f>IF(D20=0,0,D14/D20)</f>
-        <v>0.16205941193998133</v>
+        <v>0.1561650914697579</v>
       </c>
       <c r="E30" s="32">
         <f>IF(E20=0,0,E14/E20)</f>
-        <v>0.14812953004327722</v>
+        <v>0.14597593751392152</v>
       </c>
       <c r="F30" s="32">
         <f>IF(F20=0,0,F14/F20)</f>
@@ -10740,11 +10740,11 @@
       </c>
       <c r="C44" s="26">
         <f>Exchange!C16*Exchange!C17+Exchange!C20*Exchange!C18</f>
-        <v>36000</v>
+        <v>108000</v>
       </c>
       <c r="D44" s="26">
         <f>Exchange!D16*Exchange!D17+Exchange!D20*Exchange!D18</f>
-        <v>84000</v>
+        <v>90000</v>
       </c>
       <c r="E44" s="26">
         <f>Exchange!E16*Exchange!E17+Exchange!E20*Exchange!E18</f>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="F44" s="26">
         <f>Exchange!F16*Exchange!F17+Exchange!F20*Exchange!F18</f>
-        <v>216000</v>
+        <v>192000</v>
       </c>
       <c r="G44" s="7" t="n"/>
     </row>
@@ -10796,11 +10796,11 @@
       </c>
       <c r="C46" s="28">
         <f>SUM(C39:C45)</f>
-        <v>174975.0</v>
+        <v>246975.0</v>
       </c>
       <c r="D46" s="28">
         <f>SUM(D39:D45)</f>
-        <v>321450.0</v>
+        <v>327450.0</v>
       </c>
       <c r="E46" s="28">
         <f>SUM(E39:E45)</f>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="F46" s="28">
         <f>SUM(F39:F45)</f>
-        <v>575000.0</v>
+        <v>551000.0</v>
       </c>
       <c r="G46" s="7" t="n"/>
     </row>
@@ -11244,15 +11244,15 @@
       </c>
       <c r="C62" s="26">
         <f>Garden!C43+Garden!C44+Exchange!C54+Exchange!C55</f>
-        <v>12726.66864</v>
+        <v>18624.844128</v>
       </c>
       <c r="D62" s="26">
         <f>Garden!D43+Garden!D44+Exchange!D54+Exchange!D55</f>
-        <v>48205.799232</v>
+        <v>56386.833216</v>
       </c>
       <c r="E62" s="26">
         <f>Garden!E43+Garden!E44+Exchange!E54+Exchange!E55</f>
-        <v>125747.647488</v>
+        <v>134539.55788799998</v>
       </c>
       <c r="F62" s="26">
         <f>Garden!F43+Garden!F44+Exchange!F54+Exchange!F55</f>
@@ -11272,15 +11272,15 @@
       </c>
       <c r="C63" s="28">
         <f>C62</f>
-        <v>12726.66864</v>
+        <v>18624.844128</v>
       </c>
       <c r="D63" s="28">
         <f>D62</f>
-        <v>48205.799232</v>
+        <v>56386.833216</v>
       </c>
       <c r="E63" s="28">
         <f>E62</f>
-        <v>125747.647488</v>
+        <v>134539.55788799998</v>
       </c>
       <c r="F63" s="28">
         <f>F62</f>
@@ -11309,19 +11309,19 @@
       </c>
       <c r="C65" s="28">
         <f>C38+C46+C49+C55+C61+C63</f>
-        <v>459026.66864</v>
+        <v>536924.844128</v>
       </c>
       <c r="D65" s="28">
         <f>D38+D46+D49+D55+D61+D63</f>
-        <v>779325.799232</v>
+        <v>793506.833216</v>
       </c>
       <c r="E65" s="28">
         <f>E38+E46+E49+E55+E61+E63</f>
-        <v>1066747.647488</v>
+        <v>1075539.557888</v>
       </c>
       <c r="F65" s="28">
         <f>F38+F46+F49+F55+F61+F63</f>
-        <v>1438856.398144</v>
+        <v>1414856.398144</v>
       </c>
       <c r="G65" s="7" t="n"/>
     </row>
@@ -11393,19 +11393,19 @@
       </c>
       <c r="C68" s="32">
         <f>IF(C65=0,0,C66/C65)</f>
-        <v>0.566198039800235</v>
+        <v>0.4840528480705602</v>
       </c>
       <c r="D68" s="32">
         <f>IF(D65=0,0,D66/D65)</f>
-        <v>0.529945242935622</v>
+        <v>0.5204744089299828</v>
       </c>
       <c r="E68" s="32">
         <f>IF(E65=0,0,E66/E65)</f>
-        <v>0.4387166928392636</v>
+        <v>0.43513043901332227</v>
       </c>
       <c r="F68" s="32">
         <f>IF(F65=0,0,F66/F65)</f>
-        <v>0.35027817970585273</v>
+        <v>0.3562198967055202</v>
       </c>
       <c r="G68" s="7" t="n"/>
     </row>
@@ -11443,19 +11443,19 @@
       </c>
       <c r="C71" s="28">
         <f>C14-C65</f>
-        <v>-312691.20944</v>
+        <v>-364645.500128</v>
       </c>
       <c r="D71" s="28">
         <f>D14-D65</f>
-        <v>-317853.274432</v>
+        <v>-294042.462016</v>
       </c>
       <c r="E71" s="28">
         <f>E14-E65</f>
-        <v>-3340.8154880001675</v>
+        <v>30067.11411199998</v>
       </c>
       <c r="F71" s="28">
         <f>F14-F65</f>
-        <v>671797.7138560002</v>
+        <v>695797.7138560002</v>
       </c>
       <c r="G71" s="7" t="n"/>
     </row>
@@ -11471,19 +11471,19 @@
       </c>
       <c r="C72" s="33">
         <f>B72+C71</f>
-        <v>-504685.077578</v>
+        <v>-556639.368266</v>
       </c>
       <c r="D72" s="33">
         <f>C72+D71</f>
-        <v>-822538.35201</v>
+        <v>-850681.8302819999</v>
       </c>
       <c r="E72" s="33">
         <f>D72+E71</f>
-        <v>-825879.1674980002</v>
+        <v>-820614.7161699999</v>
       </c>
       <c r="F72" s="33">
         <f>E72+F71</f>
-        <v>-154081.45364199998</v>
+        <v>-124817.00231399969</v>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
@@ -11499,7 +11499,7 @@
       </c>
       <c r="B73" s="28">
         <f>-MIN(0,MIN(B72:F72))</f>
-        <v>825879.1674980002</v>
+        <v>850681.8302819999</v>
       </c>
       <c r="C73" s="28" t="inlineStr"/>
       <c r="D73" s="28" t="inlineStr"/>
@@ -11551,15 +11551,15 @@
       </c>
       <c r="C75" s="27">
         <f>C14/C74</f>
-        <v>48778.486399999994</v>
+        <v>57426.448</v>
       </c>
       <c r="D75" s="27">
         <f>D14/D74</f>
-        <v>115368.1312</v>
+        <v>124866.0928</v>
       </c>
       <c r="E75" s="27">
         <f>E14/E74</f>
-        <v>265851.708</v>
+        <v>276401.668</v>
       </c>
       <c r="F75" s="27">
         <f>F14/F74</f>
@@ -11992,7 +11992,7 @@
       </c>
       <c r="B31" s="29">
         <f>Combined!D21</f>
-        <v>7620</v>
+        <v>8580</v>
       </c>
       <c r="C31" s="8" t="inlineStr"/>
     </row>
@@ -12004,7 +12004,7 @@
       </c>
       <c r="B32" s="32">
         <f>B31/B22</f>
-        <v>0.21598639455782312</v>
+        <v>0.24319727891156462</v>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
@@ -12306,7 +12306,7 @@
       </c>
       <c r="C11" s="39">
         <f>IF(B17=0,0,B11/B17)</f>
-        <v>0.3669765980900019</v>
+        <v>0.33819570008132177</v>
       </c>
       <c r="D11" s="26">
         <f>Combined!B38</f>
@@ -12338,11 +12338,11 @@
       </c>
       <c r="B12" s="26">
         <f>Combined!B46*$B$6+Combined!C46*$B$7</f>
-        <v>166047.5</v>
+        <v>202047.5</v>
       </c>
       <c r="C12" s="39">
         <f>IF(B17=0,0,B12/B17)</f>
-        <v>0.3628033679433761</v>
+        <v>0.4068386092444866</v>
       </c>
       <c r="D12" s="26">
         <f>Combined!B46</f>
@@ -12350,11 +12350,11 @@
       </c>
       <c r="E12" s="26">
         <f>Combined!C46</f>
-        <v>174975.0</v>
+        <v>246975.0</v>
       </c>
       <c r="F12" s="26">
         <f>Combined!D46</f>
-        <v>321450.0</v>
+        <v>327450.0</v>
       </c>
       <c r="G12" s="26">
         <f>Combined!E46</f>
@@ -12378,7 +12378,7 @@
       </c>
       <c r="C13" s="39">
         <f>IF(B17=0,0,B13/B17)</f>
-        <v>0.010924686247711531</v>
+        <v>0.010067895154468296</v>
       </c>
       <c r="D13" s="26">
         <f>Combined!B49</f>
@@ -12414,7 +12414,7 @@
       </c>
       <c r="C14" s="39">
         <f>IF(B17=0,0,B14/B17)</f>
-        <v>0.164929988281701</v>
+        <v>0.1519950131470079</v>
       </c>
       <c r="D14" s="26">
         <f>Combined!B55</f>
@@ -12450,7 +12450,7 @@
       </c>
       <c r="C15" s="39">
         <f>IF(B17=0,0,B15/B17)</f>
-        <v>0.07538033510920956</v>
+        <v>0.06946847656583124</v>
       </c>
       <c r="D15" s="26">
         <f>Combined!B61</f>
@@ -12482,11 +12482,11 @@
       </c>
       <c r="B16" s="26">
         <f>Combined!B63*$B$6+Combined!C63*$B$7</f>
-        <v>8689.047858</v>
+        <v>11638.135602</v>
       </c>
       <c r="C16" s="39">
         <f>IF(B17=0,0,B16/B17)</f>
-        <v>0.018985024327999988</v>
+        <v>0.023434305806884156</v>
       </c>
       <c r="D16" s="26">
         <f>Combined!B63</f>
@@ -12494,15 +12494,15 @@
       </c>
       <c r="E16" s="26">
         <f>Combined!C63</f>
-        <v>12726.66864</v>
+        <v>18624.844128</v>
       </c>
       <c r="F16" s="26">
         <f>Combined!D63</f>
-        <v>48205.799232</v>
+        <v>56386.833216</v>
       </c>
       <c r="G16" s="26">
         <f>Combined!E63</f>
-        <v>125747.647488</v>
+        <v>134539.55788799998</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
@@ -12518,7 +12518,7 @@
       </c>
       <c r="B17" s="33">
         <f>SUM(B11:B16)</f>
-        <v>457679.047858</v>
+        <v>496628.135602</v>
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="33">
@@ -12527,15 +12527,15 @@
       </c>
       <c r="E17" s="33">
         <f>SUM(E11:E16)</f>
-        <v>459026.66864</v>
+        <v>536924.844128</v>
       </c>
       <c r="F17" s="33">
         <f>SUM(F11:F16)</f>
-        <v>779325.799232</v>
+        <v>793506.833216</v>
       </c>
       <c r="G17" s="33">
         <f>SUM(G11:G16)</f>
-        <v>1066747.647488</v>
+        <v>1075539.557888</v>
       </c>
       <c r="H17" s="7" t="n"/>
     </row>
@@ -12551,7 +12551,7 @@
       </c>
       <c r="C18" s="39">
         <f>IF(B17=0,0,B18/B17)</f>
-        <v>0.44559610267165795</v>
+        <v>0.41064930756045287</v>
       </c>
       <c r="D18" s="26">
         <f>Combined!B67</f>
@@ -12670,7 +12670,7 @@
       </c>
       <c r="C22" s="39">
         <f>IF(B17=0,0,B22/B17)</f>
-        <v>0.5794235092061242</v>
+        <v>0.5339810232026895</v>
       </c>
       <c r="D22" s="26">
         <f>Combined!B66</f>
@@ -12708,7 +12708,7 @@
       </c>
       <c r="B24" s="26">
         <f>Combined!B14*$B$6+Combined!C14*$B$7</f>
-        <v>109339.575</v>
+        <v>122311.5174</v>
       </c>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="26">
@@ -12717,15 +12717,15 @@
       </c>
       <c r="E24" s="26">
         <f>Combined!C14</f>
-        <v>146335.45919999998</v>
+        <v>172279.34399999998</v>
       </c>
       <c r="F24" s="26">
         <f>Combined!D14</f>
-        <v>461472.5248</v>
+        <v>499464.3712</v>
       </c>
       <c r="G24" s="26">
         <f>Combined!E14</f>
-        <v>1063406.832</v>
+        <v>1105606.672</v>
       </c>
       <c r="H24" s="7" t="n"/>
     </row>
@@ -12737,7 +12737,7 @@
       </c>
       <c r="B25" s="33">
         <f>B17-B24</f>
-        <v>348339.47285799996</v>
+        <v>374316.618202</v>
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
@@ -12754,11 +12754,11 @@
       </c>
       <c r="B26" s="33">
         <f>B4-B25</f>
-        <v>1660.5271420000354</v>
+        <v>-24316.618201999983</v>
       </c>
       <c r="C26" s="39">
         <f>IF(B25=0,0,B26/B25)</f>
-        <v>0.004766979545487647</v>
+        <v>-0.06496270007675031</v>
       </c>
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
@@ -13040,15 +13040,15 @@
       </c>
       <c r="E37" s="42">
         <f>IF(E36=0,0,Combined!C14/E36)</f>
-        <v>48778.486399999994</v>
+        <v>57426.448</v>
       </c>
       <c r="F37" s="42">
         <f>IF(F36=0,0,Combined!D14/F36)</f>
-        <v>115368.1312</v>
+        <v>124866.0928</v>
       </c>
       <c r="G37" s="42">
         <f>IF(G36=0,0,Combined!E14/G36)</f>
-        <v>265851.708</v>
+        <v>276401.668</v>
       </c>
       <c r="H37" s="42">
         <f>IF(H36=0,0,Combined!F14/H36)</f>
@@ -13121,15 +13121,15 @@
       </c>
       <c r="C41" s="26">
         <f>MAX(0,Combined!C65-Combined!C14)</f>
-        <v>312691.20944</v>
+        <v>364645.500128</v>
       </c>
       <c r="D41" s="26">
         <f>MAX(0,Combined!D65-Combined!D14)</f>
-        <v>317853.274432</v>
+        <v>294042.462016</v>
       </c>
       <c r="E41" s="26">
         <f>MAX(0,Combined!E65-Combined!E14)</f>
-        <v>3340.8154880001675</v>
+        <v>0</v>
       </c>
       <c r="F41" s="26">
         <f>MAX(0,Combined!F65-Combined!F14)</f>
@@ -13150,15 +13150,15 @@
       </c>
       <c r="C42" s="42">
         <f>C41/12</f>
-        <v>26057.600786666666</v>
+        <v>30387.125010666667</v>
       </c>
       <c r="D42" s="42">
         <f>D41/12</f>
-        <v>26487.772869333334</v>
+        <v>24503.538501333333</v>
       </c>
       <c r="E42" s="42">
         <f>E41/12</f>
-        <v>278.4012906666806</v>
+        <v>0.0</v>
       </c>
       <c r="F42" s="42">
         <f>F41/12</f>
@@ -13224,7 +13224,7 @@
       </c>
       <c r="B46" s="44">
         <f>MIN(60,IF(A46&lt;=$B$41,A46/MAX(1,$B$41/12),IF(A46&lt;=$B$41+$C$41,12+(A46-$B$41)/MAX(1,$C$41/12),IF(A46&lt;=$B$41+$C$41+$D$41,24+(A46-$B$41-$C$41)/MAX(1,$D$41/12),IF(A46&lt;=$B$41+$C$41+$D$41+$E$41,36+(A46-$B$41-$C$41-$D$41)/MAX(1,$E$41/12),IF(A46&lt;=$B$41+$C$41+$D$41+$E$41+$F$41,48+(A46-$B$41-$C$41-$D$41-$E$41)/MAX(1,$F$41/12),60))))))</f>
-        <v>14.226073395509266</v>
+        <v>13.90890490106051</v>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
@@ -13243,7 +13243,7 @@
       </c>
       <c r="B47" s="44">
         <f>MIN(60,IF(A47&lt;=$B$41,A47/MAX(1,$B$41/12),IF(A47&lt;=$B$41+$C$41,12+(A47-$B$41)/MAX(1,$C$41/12),IF(A47&lt;=$B$41+$C$41+$D$41,24+(A47-$B$41-$C$41)/MAX(1,$D$41/12),IF(A47&lt;=$B$41+$C$41+$D$41+$E$41,36+(A47-$B$41-$C$41-$D$41)/MAX(1,$E$41/12),IF(A47&lt;=$B$41+$C$41+$D$41+$E$41+$F$41,48+(A47-$B$41-$C$41-$D$41-$E$41)/MAX(1,$F$41/12),60))))))</f>
-        <v>18.063725250670416</v>
+        <v>17.199772331424434</v>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
@@ -13262,7 +13262,7 @@
       </c>
       <c r="B48" s="44">
         <f>MIN(60,IF(A48&lt;=$B$41,A48/MAX(1,$B$41/12),IF(A48&lt;=$B$41+$C$41,12+(A48-$B$41)/MAX(1,$C$41/12),IF(A48&lt;=$B$41+$C$41+$D$41,24+(A48-$B$41-$C$41)/MAX(1,$D$41/12),IF(A48&lt;=$B$41+$C$41+$D$41+$E$41,36+(A48-$B$41-$C$41-$D$41)/MAX(1,$E$41/12),IF(A48&lt;=$B$41+$C$41+$D$41+$E$41+$F$41,48+(A48-$B$41-$C$41-$D$41-$E$41)/MAX(1,$F$41/12),60))))))</f>
-        <v>23.82020303341214</v>
+        <v>22.136073476970324</v>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="B49" s="44">
         <f>MIN(60,IF(A49&lt;=$B$41,A49/MAX(1,$B$41/12),IF(A49&lt;=$B$41+$C$41,12+(A49-$B$41)/MAX(1,$C$41/12),IF(A49&lt;=$B$41+$C$41+$D$41,24+(A49-$B$41-$C$41)/MAX(1,$D$41/12),IF(A49&lt;=$B$41+$C$41+$D$41+$E$41,36+(A49-$B$41-$C$41-$D$41)/MAX(1,$E$41/12),IF(A49&lt;=$B$41+$C$41+$D$41+$E$41+$F$41,48+(A49-$B$41-$C$41-$D$41-$E$41)/MAX(1,$F$41/12),60))))))</f>
-        <v>29.48611327720349</v>
+        <v>27.810087744221917</v>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
@@ -13300,7 +13300,7 @@
       </c>
       <c r="B50" s="44">
         <f>MIN(60,IF(A50&lt;=$B$41,A50/MAX(1,$B$41/12),IF(A50&lt;=$B$41+$C$41,12+(A50-$B$41)/MAX(1,$C$41/12),IF(A50&lt;=$B$41+$C$41+$D$41,24+(A50-$B$41-$C$41)/MAX(1,$D$41/12),IF(A50&lt;=$B$41+$C$41+$D$41+$E$41,36+(A50-$B$41-$C$41-$D$41)/MAX(1,$E$41/12),IF(A50&lt;=$B$41+$C$41+$D$41+$E$41+$F$41,48+(A50-$B$41-$C$41-$D$41-$E$41)/MAX(1,$F$41/12),60))))))</f>
-        <v>35.14910354595746</v>
+        <v>33.931652594614356</v>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
@@ -13407,7 +13407,7 @@
       </c>
       <c r="B4" s="24">
         <f>Combined!D21</f>
-        <v>7620</v>
+        <v>8580</v>
       </c>
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="7" t="n"/>
@@ -13424,7 +13424,7 @@
       </c>
       <c r="B5" s="45">
         <f>Combined!D29</f>
-        <v>60.56069879265092</v>
+        <v>58.212630675990674</v>
       </c>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="B6" s="26">
         <f>Combined!D65</f>
-        <v>779325.799232</v>
+        <v>793506.833216</v>
       </c>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="7" t="n"/>

</xml_diff>

<commit_message>
Deck and model: three-person team (two full time, one part time); Rick's phone on the team slide
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETG5M27XfcTD2TyhhuebtG
</commit_message>
<xml_diff>
--- a/docs/financial-model-5yr-v2.xlsx
+++ b/docs/financial-model-5yr-v2.xlsx
@@ -634,7 +634,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>4. Results (2026-10-01: metros as explicit drivers, a Base team of four, founder pay inside the functions). Base revenue $36k / $172k / $499k / $1.11M / $2.11M; EBITDA -$192k / -$365k / -$294k / +$30k / +$696k, so breakeven in year four and about $851k of cumulative capital at the low point, in year three. Fundable revenue $80k / $363k / $1.38M / $3.89M / $9.29M with 40 metros and a team of 18, EBITDA positive in year four. Conservative: $17k growing to $313k with 5 metros, not profitable in five years. Costs, EBITDA and cash are on the Combined sheet; docs/funding/cfo-memo-ask-and-spend.md carries the discussion.</t>
+          <t>4. Results (2026-10-01: metros as explicit drivers, a Base team of two full-time founders and one part-time founder (unpaid in the plan), plus two hires, founder pay inside the functions). Base revenue $36k / $172k / $499k / $1.11M / $2.11M; EBITDA -$192k / -$365k / -$294k / +$30k / +$696k, so breakeven in year four and about $851k of cumulative capital at the low point, in year three. Fundable revenue $80k / $363k / $1.38M / $3.89M / $9.29M with 40 metros and a team of 18, EBITDA positive in year four. Conservative: $17k growing to $313k with 5 metros, not profitable in five years. Costs, EBITDA and cash are on the Combined sheet; docs/funding/cfo-memo-ask-and-spend.md carries the discussion.</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="H171" s="8" t="inlineStr">
         <is>
-          <t>No full-time employee before both founders are full time. Base is a four-person company: one community &amp; partnerships lead from month 18 (half time in Y2, full from Y3); metros run themselves</t>
+          <t>No full-time employee before both founders are full time. Base is two full-time founders plus one part-time founder (Patricia Sinay, no pay in the model) and two hires: one community &amp; partnerships lead from month 18 (half time in Y2, full from Y3); metros run themselves</t>
         </is>
       </c>
     </row>
@@ -12831,7 +12831,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Founders (Rick: product &amp; engineering; Haley: community &amp; programs)</t>
+          <t>Full-time founders (Rick: product &amp; engineering; Haley: chief creative &amp; programs)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n"/>
@@ -13086,14 +13086,28 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n"/>
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>Part-time founder (Patricia Sinay, civic partnerships): people, not in FTE or cost</t>
+        </is>
+      </c>
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
+      <c r="D39" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="40" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">

</xml_diff>